<commit_message>
feat(mobile): real estate (buy vs rent, true cost, rental yield); tracker marks the redirect calculators done
- lib/realEstate.ts: port of js/finos-real-estate.js; parity test runs the
  website module on 600 random scenarios (0% loan, no loan, short tenure,
  tax claim) plus true cost and rental yield.
- app/tools/realestate.tsx: three tabs, inputs remembered on the device,
  the winner, both net worths, break-even, the detail, and what it assumes.
  Linked from the dashboard and the calculators hub.
- Tracker: 14 website calculator pages that only redirect to a full tool
  are marked Done with the phone screen that covers them; SIP Optimizer is
  Not planned (unseeded Math.random Monte Carlo with a fixed fund list).
  Real estate rows done. Docs and test count (290).
</commit_message>
<xml_diff>
--- a/docs/MOBILE_PARITY_TRACKER.xlsx
+++ b/docs/MOBILE_PARITY_TRACKER.xlsx
@@ -2486,7 +2486,7 @@
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
@@ -2502,13 +2502,17 @@
       <c r="H26" s="30" t="n"/>
       <c r="I26" s="30" t="inlineStr">
         <is>
-          <t>tools/real-estate</t>
-        </is>
-      </c>
-      <c r="J26" s="30" t="n"/>
+          <t>app/tools/realestate.tsx</t>
+        </is>
+      </c>
+      <c r="J26" s="30" t="inlineStr">
+        <is>
+          <t>Buy vs rent (corrected like-for-like model), true cost, rental yield; shared js/finos-real-estate.js; parity-tested</t>
+        </is>
+      </c>
       <c r="K26" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -3377,7 +3381,7 @@
       </c>
       <c r="E43" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F43" s="30" t="inlineStr">
@@ -3393,17 +3397,17 @@
       <c r="H43" s="30" t="n"/>
       <c r="I43" s="30" t="inlineStr">
         <is>
-          <t>calculators/epf</t>
+          <t>app/tracker/epf.tsx</t>
         </is>
       </c>
       <c r="J43" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the EPF tracker; the phone has it</t>
         </is>
       </c>
       <c r="K43" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3487,7 @@
       </c>
       <c r="E45" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F45" s="30" t="inlineStr">
@@ -3499,17 +3503,17 @@
       <c r="H45" s="30" t="n"/>
       <c r="I45" s="30" t="inlineStr">
         <is>
-          <t>calculators/nps</t>
+          <t>app/tracker/nps.tsx</t>
         </is>
       </c>
       <c r="J45" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the NPS tracker; the phone has it</t>
         </is>
       </c>
       <c r="K45" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -3589,7 +3593,7 @@
       </c>
       <c r="E47" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F47" s="30" t="inlineStr">
@@ -3605,17 +3609,17 @@
       <c r="H47" s="30" t="n"/>
       <c r="I47" s="30" t="inlineStr">
         <is>
-          <t>calculators/ppf</t>
+          <t>app/tracker/ppf.tsx</t>
         </is>
       </c>
       <c r="J47" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the PPF tracker; the phone has it</t>
         </is>
       </c>
       <c r="K47" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -4384,7 +4388,7 @@
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
@@ -4400,17 +4404,17 @@
       <c r="H62" s="30" t="n"/>
       <c r="I62" s="30" t="inlineStr">
         <is>
-          <t>calculators/buyhouse</t>
+          <t>app/tools/realestate.tsx</t>
         </is>
       </c>
       <c r="J62" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Buy vs rent (corrected like-for-like model), true cost, rental yield; shared js/finos-real-estate.js; parity-tested</t>
         </is>
       </c>
       <c r="K62" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -4914,7 +4918,7 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
@@ -4930,17 +4934,17 @@
       <c r="H72" s="30" t="n"/>
       <c r="I72" s="30" t="inlineStr">
         <is>
-          <t>calculators/emergencyfund</t>
+          <t>app/tracker/emergency.tsx</t>
         </is>
       </c>
       <c r="J72" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the Emergency Fund tracker; the phone has it</t>
         </is>
       </c>
       <c r="K72" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -5073,7 +5077,7 @@
       </c>
       <c r="E75" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F75" s="30" t="inlineStr">
@@ -5089,17 +5093,17 @@
       <c r="H75" s="30" t="n"/>
       <c r="I75" s="30" t="inlineStr">
         <is>
-          <t>calculators/lifestyle</t>
+          <t>app/tools/calc/lifestylecreep</t>
         </is>
       </c>
       <c r="J75" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the Lifestyle Inflation Detector (desi) which is ported</t>
         </is>
       </c>
       <c r="K75" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5130,7 @@
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
@@ -5142,17 +5146,17 @@
       <c r="H76" s="30" t="n"/>
       <c r="I76" s="30" t="inlineStr">
         <is>
-          <t>calculators/networth</t>
+          <t>app/tracker/networth.tsx</t>
         </is>
       </c>
       <c r="J76" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to Net Worth; the phone has it</t>
         </is>
       </c>
       <c r="K76" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -5444,7 +5448,7 @@
       </c>
       <c r="E82" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F82" s="30" t="inlineStr">
@@ -5460,17 +5464,17 @@
       <c r="H82" s="30" t="n"/>
       <c r="I82" s="30" t="inlineStr">
         <is>
-          <t>calculators/goalbased</t>
+          <t>app/tools/goalopt.tsx</t>
         </is>
       </c>
       <c r="J82" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the Goal Optimizer; the phone has it</t>
         </is>
       </c>
       <c r="K82" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -5656,7 +5660,7 @@
       </c>
       <c r="E86" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F86" s="30" t="inlineStr">
@@ -5672,17 +5676,17 @@
       <c r="H86" s="30" t="n"/>
       <c r="I86" s="30" t="inlineStr">
         <is>
-          <t>calculators/rebalancing</t>
+          <t>app/tools/rebalance.tsx</t>
         </is>
       </c>
       <c r="J86" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the Portfolio Rebalancer; the phone has it</t>
         </is>
       </c>
       <c r="K86" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -5762,7 +5766,7 @@
       </c>
       <c r="E88" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
@@ -5783,12 +5787,12 @@
       </c>
       <c r="J88" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Random (Math.random) Monte Carlo with a fixed fund list: not reproducible and prescriptive. The Goal Optimizer and Retirement Planner (seeded) cover it</t>
         </is>
       </c>
       <c r="K88" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -5868,7 +5872,7 @@
       </c>
       <c r="E90" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
@@ -5884,17 +5888,17 @@
       <c r="H90" s="30" t="n"/>
       <c r="I90" s="30" t="inlineStr">
         <is>
-          <t>calculators/stepup</t>
+          <t>app/tools/stepup.tsx</t>
         </is>
       </c>
       <c r="J90" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the SIP Step-up planner; the phone has it</t>
         </is>
       </c>
       <c r="K90" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -6186,7 +6190,7 @@
       </c>
       <c r="E96" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F96" s="30" t="inlineStr">
@@ -6202,17 +6206,17 @@
       <c r="H96" s="30" t="n"/>
       <c r="I96" s="30" t="inlineStr">
         <is>
-          <t>calculators/debtsnow</t>
+          <t>app/tools/debt.tsx</t>
         </is>
       </c>
       <c r="J96" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the Debt Optimizer; the phone has it</t>
         </is>
       </c>
       <c r="K96" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -6398,7 +6402,7 @@
       </c>
       <c r="E100" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F100" s="30" t="inlineStr">
@@ -6414,17 +6418,17 @@
       <c r="H100" s="30" t="n"/>
       <c r="I100" s="30" t="inlineStr">
         <is>
-          <t>calculators/home</t>
+          <t>app/tools/homeloan.tsx</t>
         </is>
       </c>
       <c r="J100" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the Home Loan planner; the phone has it</t>
         </is>
       </c>
       <c r="K100" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -7034,7 +7038,7 @@
       </c>
       <c r="E112" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F112" s="30" t="inlineStr">
@@ -7050,17 +7054,17 @@
       <c r="H112" s="30" t="n"/>
       <c r="I112" s="30" t="inlineStr">
         <is>
-          <t>calculators/retirement</t>
+          <t>app/tools/retirement.tsx</t>
         </is>
       </c>
       <c r="J112" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the Retirement Planner; the phone has it</t>
         </is>
       </c>
       <c r="K112" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -7299,7 +7303,7 @@
       </c>
       <c r="E117" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F117" s="30" t="inlineStr">
@@ -7315,17 +7319,17 @@
       <c r="H117" s="30" t="n"/>
       <c r="I117" s="30" t="inlineStr">
         <is>
-          <t>calculators/income</t>
+          <t>app/tools/taxplanner.tsx</t>
         </is>
       </c>
       <c r="J117" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Uses the shared tax core; the phone Tax Planner compares both regimes on the same port</t>
         </is>
       </c>
       <c r="K117" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -7352,7 +7356,7 @@
       </c>
       <c r="E118" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F118" s="30" t="inlineStr">
@@ -7368,17 +7372,17 @@
       <c r="H118" s="30" t="n"/>
       <c r="I118" s="30" t="inlineStr">
         <is>
-          <t>calculators/inhand</t>
+          <t>app/tools/salary.tsx</t>
         </is>
       </c>
       <c r="J118" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Website page redirects to the Salary Optimizer; the phone has it</t>
         </is>
       </c>
       <c r="K118" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -7511,7 +7515,7 @@
       </c>
       <c r="E121" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F121" s="30" t="inlineStr">
@@ -7527,17 +7531,17 @@
       <c r="H121" s="30" t="n"/>
       <c r="I121" s="30" t="inlineStr">
         <is>
-          <t>calculators/oldnew</t>
+          <t>app/tools/taxplanner.tsx</t>
         </is>
       </c>
       <c r="J121" s="30" t="inlineStr">
         <is>
-          <t>Pure formula; port + parity test</t>
+          <t>Old vs new regime: the phone Tax Planner (parity-tested on the shared tax core)</t>
         </is>
       </c>
       <c r="K121" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
     </row>
@@ -15032,7 +15036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="16" min="1" max="1"/>
@@ -15734,28 +15738,53 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>2026-10-14</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
         <is>
           <t>C-01…C-90 (71 of 88)</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
+      <c r="C27" s="16" t="inlineStr">
         <is>
           <t>Calculators hub + 71 calculators across 9 groups; parity harness runs each website page script; 3 website bugs found and fixed (SSY double count, Options zero-strike hang, Bond coupon float)</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
+      <c r="D27" s="16" t="inlineStr">
         <is>
           <t>webCalc.parity.test.mts: 63 pages x ~70 vectors each; preview run</t>
         </is>
       </c>
-      <c r="E27" t="n">
+      <c r="E27" s="16" t="n">
         <v>287</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>T-25, C-21</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Real estate: buy vs rent, true cost, rental yield on the phone; website page rewired to a shared tested module with a corrected model</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>tests/real-estate.test.js (11), test_real_estate_ui.py (4), realEstate.parity (3); preview run</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>290</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Mobile polish: cross-links, honest Home greeting and strip, no assumed ages, Hindi first pass, release docs
- Budget to Forecast, Goals to Life goals, Portfolio to Growth, Insurance tracker to hub, Watchlist rows to research,
  feedback prompt on the Money Score result
- Home: greeting names the person only when a name is recorded, N-day streak, strip of savings rate / net worth /
  Money Score from recorded facts, hideable (Settings brings it back)
- an unknown age is never replaced by 30 (insurance gaps, Money Score, PULSE, life events); privacy notice says an
  unreadable value is kept on the phone until erase, with a guard test
- Budget / Goals inputs no longer clip long figures; Portfolio header wraps; smoke script now renders populated Portfolio
- Hindi: about 200 short first-pass entries (unreviewed)
- runbook and device checklist brought up to date; parity tracker rows audited against the code; build log extended
</commit_message>
<xml_diff>
--- a/docs/MOBILE_PARITY_TRACKER.xlsx
+++ b/docs/MOBILE_PARITY_TRACKER.xlsx
@@ -664,10 +664,11 @@
     <row r="2" ht="15" customHeight="1" s="17">
       <c r="A2" s="19" t="inlineStr">
         <is>
-          <t>Source of truth: the 'Parity Tracker' sheet. Counts below are formulas. Last built 2026-10-12.</t>
-        </is>
-      </c>
-    </row>
+          <t>Source of truth: the 'Parity Tracker' sheet. Counts below are formulas. All rows audited against the code and the agent notes on 2026-10-17 (final integration). Nothing is marked as verified on a device: every status rests on the Expo web preview and unit tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
     <row r="4" ht="15" customHeight="1" s="17">
       <c r="A4" s="20" t="inlineStr">
         <is>
@@ -9231,7 +9232,7 @@
       </c>
       <c r="E153" s="30" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F153" s="30" t="inlineStr">
@@ -9252,12 +9253,12 @@
       </c>
       <c r="J153" s="30" t="inlineStr">
         <is>
-          <t>Interactive page: not flattened into text. It has no phone equivalent, so the lesson screen says it is interactive on the website.</t>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a menu page on the website: the phone page lists its five entries, each mapped to a lesson, tool or tab. Web preview only. Not verified on a device.</t>
         </is>
       </c>
       <c r="K153" s="30" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9337,7 +9338,7 @@
       </c>
       <c r="E155" s="30" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F155" s="30" t="inlineStr">
@@ -9358,12 +9359,12 @@
       </c>
       <c r="J155" s="30" t="inlineStr">
         <is>
-          <t>Interactive page: not flattened into text. The lesson screen links to the matching phone tool: Financial DNA (/tools/dna).</t>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): demonstration panels with example numbers ("Simulated sector momentum scores"); not flattened. The page says so and points to Financial DNA, which is a different tool. Not verified on a device.</t>
         </is>
       </c>
       <c r="K155" s="30" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9390,7 +9391,7 @@
       </c>
       <c r="E156" s="30" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F156" s="30" t="inlineStr">
@@ -9411,12 +9412,12 @@
       </c>
       <c r="J156" s="30" t="inlineStr">
         <is>
-          <t>Interactive page: not flattened into text. The lesson screen links to the matching phone tool: Financial DNA (/tools/dna).</t>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): an imagined "Indian market translation" of ten investors; not copied. The page says so and points to Financial DNA, a different tool. Not verified on a device.</t>
         </is>
       </c>
       <c r="K156" s="30" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9492,7 +9493,7 @@
       </c>
       <c r="E158" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F158" s="30" t="inlineStr">
@@ -9511,10 +9512,14 @@
           <t>learn/mindset-sim</t>
         </is>
       </c>
-      <c r="J158" s="30" t="n"/>
+      <c r="J158" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): the 20 scenarios as case studies (Hinglish as on the website), each passage with its source line. The choose-then-reveal flow, score and AI debrief are not on the phone and the lesson says so. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K158" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9541,7 +9546,7 @@
       </c>
       <c r="E159" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F159" s="30" t="inlineStr">
@@ -9560,10 +9565,14 @@
           <t>learn/mindset-sim-hub</t>
         </is>
       </c>
-      <c r="J159" s="30" t="n"/>
+      <c r="J159" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): the website page only forwards to the Simulator Hub; the phone page says so. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K159" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9590,7 +9599,7 @@
       </c>
       <c r="E160" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F160" s="30" t="inlineStr">
@@ -9609,10 +9618,14 @@
           <t>learn/train-mindset</t>
         </is>
       </c>
-      <c r="J160" s="30" t="n"/>
+      <c r="J160" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): the website page only forwards to the Simulator Hub; the phone page says so. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K160" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9639,7 +9652,7 @@
       </c>
       <c r="E161" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F161" s="30" t="inlineStr">
@@ -9658,10 +9671,14 @@
           <t>learn/not-money</t>
         </is>
       </c>
-      <c r="J161" s="30" t="n"/>
+      <c r="J161" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): the website page only forwards to the AI Mindset Simulator; the phone page says so. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K161" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9688,7 +9705,7 @@
       </c>
       <c r="E162" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F162" s="30" t="inlineStr">
@@ -9707,10 +9724,14 @@
           <t>learn/decision</t>
         </is>
       </c>
-      <c r="J162" s="30" t="n"/>
+      <c r="J162" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): lesson text (fast vs slow thinking, three biases, checklist). The doughnut chart of fixed example slices is left out and said so. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K162" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9737,7 +9758,7 @@
       </c>
       <c r="E163" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F163" s="30" t="inlineStr">
@@ -9756,10 +9777,14 @@
           <t>learn/clarity</t>
         </is>
       </c>
-      <c r="J163" s="30" t="n"/>
+      <c r="J163" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): lesson text plus a link to Net worth. The scanner strip, DONE/CURRENT/LOCKED labels and the EMI slider (rough x120x1.8 rule) are not shown; each is explained. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K163" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9786,7 +9811,7 @@
       </c>
       <c r="E164" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F164" s="30" t="inlineStr">
@@ -9805,10 +9830,14 @@
           <t>learn/scenarios</t>
         </is>
       </c>
-      <c r="J164" s="30" t="n"/>
+      <c r="J164" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a hub: the nine what-if simulations run on stored numbers with AI narration on the website and are not on the phone; each is listed with the closest phone tool (or none). Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K164" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9835,7 +9864,7 @@
       </c>
       <c r="E165" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F165" s="30" t="inlineStr">
@@ -9854,10 +9883,14 @@
           <t>learn/timeline</t>
         </is>
       </c>
-      <c r="J165" s="30" t="n"/>
+      <c r="J165" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): the website page shows generated sample scores whenever it cannot reach its alert service, so it was not copied. The phone page explains this and names Money Score as the nearest real thing. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K165" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9884,7 +9917,7 @@
       </c>
       <c r="E166" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F166" s="30" t="inlineStr">
@@ -9903,10 +9936,14 @@
           <t>learn/fear-roadmap</t>
         </is>
       </c>
-      <c r="J166" s="30" t="n"/>
+      <c r="J166" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a quiz whose answers pick written outcomes, so not lesson text for everyone; the page explains why there is no honest equivalent. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K166" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9933,7 +9970,7 @@
       </c>
       <c r="E167" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F167" s="30" t="inlineStr">
@@ -9952,10 +9989,14 @@
           <t>learn/roadmap</t>
         </is>
       </c>
-      <c r="J167" s="30" t="n"/>
+      <c r="J167" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a hub: the personalised roadmap and mind map are built from stored data on the website and are not on the phone; its 7-path menu is listed with the phone equivalents (e.g. Arya Plan). Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K167" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -9982,7 +10023,7 @@
       </c>
       <c r="E168" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F168" s="30" t="inlineStr">
@@ -10001,10 +10042,14 @@
           <t>learn/roadmaps</t>
         </is>
       </c>
-      <c r="J168" s="30" t="n"/>
+      <c r="J168" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): the website page only redirects to Roadmap; the phone page says so. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K168" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10031,7 +10076,7 @@
       </c>
       <c r="E169" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F169" s="30" t="inlineStr">
@@ -10050,10 +10095,14 @@
           <t>learn/trader-roadmap</t>
         </is>
       </c>
-      <c r="J169" s="30" t="n"/>
+      <c r="J169" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a six-question quiz that picks one of five personas (one says to close all trading accounts), so not general advice; the page explains why there is no honest equivalent. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K169" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10080,7 +10129,7 @@
       </c>
       <c r="E170" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F170" s="30" t="inlineStr">
@@ -10099,10 +10148,14 @@
           <t>learn/traditional-roadmap</t>
         </is>
       </c>
-      <c r="J170" s="30" t="n"/>
+      <c r="J170" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a two-question quiz whose step list has out-of-date tax and inflation statements; not copied, the page explains why. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K170" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10129,7 +10182,7 @@
       </c>
       <c r="E171" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F171" s="30" t="inlineStr">
@@ -10148,10 +10201,14 @@
           <t>learn/simulator</t>
         </is>
       </c>
-      <c r="J171" s="30" t="n"/>
+      <c r="J171" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): the website page only redirects to the Simulator Hub; the phone page says so. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K171" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10231,7 +10288,7 @@
       </c>
       <c r="E173" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F173" s="30" t="inlineStr">
@@ -10250,10 +10307,14 @@
           <t>learn/simulator-landing</t>
         </is>
       </c>
-      <c r="J173" s="30" t="n"/>
+      <c r="J173" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a hub: menu of six simulator cards (the ticker strip uses fixed typed-in prices and is not shown); the simulators themselves are not on the phone. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K173" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10280,7 +10341,7 @@
       </c>
       <c r="E174" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F174" s="30" t="inlineStr">
@@ -10299,10 +10360,14 @@
           <t>learn/trading-simulator</t>
         </is>
       </c>
-      <c r="J174" s="30" t="n"/>
+      <c r="J174" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): website only: a practice-trading UI with generated candles. No trading features on the phone; the phone page says so. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K174" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10329,7 +10394,7 @@
       </c>
       <c r="E175" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F175" s="30" t="inlineStr">
@@ -10348,10 +10413,14 @@
           <t>learn/trading-coach</t>
         </is>
       </c>
-      <c r="J175" s="30" t="n"/>
+      <c r="J175" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a 3-question clearance plus an AI assessment; trader-only and needs the website AI service. The page explains why. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K175" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10378,7 +10447,7 @@
       </c>
       <c r="E176" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F176" s="30" t="inlineStr">
@@ -10397,10 +10466,14 @@
           <t>learn/trading-brain</t>
         </is>
       </c>
-      <c r="J176" s="30" t="n"/>
+      <c r="J176" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): live signals from data services, and pattern tables quote win rates with no stated method; not copied. The page explains why. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K176" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10427,7 +10500,7 @@
       </c>
       <c r="E177" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F177" s="30" t="inlineStr">
@@ -10446,10 +10519,14 @@
           <t>learn/know-your-finances</t>
         </is>
       </c>
-      <c r="J177" s="30" t="n"/>
+      <c r="J177" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a long input form plus an AI scan; the page explains why and names the phone parts (Net worth, Money Score, Retirement planner). Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K177" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10476,7 +10553,7 @@
       </c>
       <c r="E178" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F178" s="30" t="inlineStr">
@@ -10495,10 +10572,14 @@
           <t>learn/financial-being</t>
         </is>
       </c>
-      <c r="J178" s="30" t="n"/>
+      <c r="J178" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a long self-assessment ending in an AI report; the page explains why and names Financial DNA as a different, shorter quiz. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K178" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10525,7 +10606,7 @@
       </c>
       <c r="E179" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F179" s="30" t="inlineStr">
@@ -10544,10 +10625,14 @@
           <t>learn/diagnostics</t>
         </is>
       </c>
-      <c r="J179" s="30" t="n"/>
+      <c r="J179" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a hub: menu of two scans and four tools; the phone has Financial DNA, Benchmarks and Future loss (not the phone's crash-notes Diagnostics screen). Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K179" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10574,7 +10659,7 @@
       </c>
       <c r="E180" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F180" s="30" t="inlineStr">
@@ -10593,10 +10678,14 @@
           <t>learn/life-wealth</t>
         </is>
       </c>
-      <c r="J180" s="30" t="n"/>
+      <c r="J180" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): lesson text (milestones and money-vs-soul pairs from the page and its script), source lines on every passage. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K180" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10623,7 +10712,7 @@
       </c>
       <c r="E181" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F181" s="30" t="inlineStr">
@@ -10642,10 +10731,14 @@
           <t>learn/impact</t>
         </is>
       </c>
-      <c r="J181" s="30" t="n"/>
+      <c r="J181" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): a hub: the compound box (= the SIP calculator on the phone) and eight story cards (= Impact stories, L-51). Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K181" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -10672,7 +10765,7 @@
       </c>
       <c r="E182" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F182" s="30" t="inlineStr">
@@ -10691,10 +10784,14 @@
           <t>learn/impact-detail</t>
         </is>
       </c>
-      <c r="J182" s="30" t="n"/>
+      <c r="J182" s="30" t="inlineStr">
+        <is>
+          <t>Learn wave 2 (docs/agent-notes/learn2.md): the eight five-step stories from js/impact-detail.js, with source lines; two stated figures are wrong on the website and are flagged in the lesson. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K182" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -11035,7 +11132,7 @@
       </c>
       <c r="E189" s="30" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F189" s="30" t="inlineStr">
@@ -11051,17 +11148,17 @@
       <c r="H189" s="30" t="n"/>
       <c r="I189" s="30" t="inlineStr">
         <is>
-          <t>markets/cryptodetail</t>
+          <t>market/crypto/[id]</t>
         </is>
       </c>
       <c r="J189" s="30" t="inlineStr">
         <is>
-          <t>Live prices only (app/market/crypto.tsx): no detail page, no on-chain or market-cap history.</t>
+          <t>portfolio-analytics.md: detail with price history. Polygon has no history source (shows today's price and says why). Chart steps on sub-5 prices (backend rounding, U14). Web preview only. Not verified on a device.</t>
         </is>
       </c>
       <c r="K189" s="30" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -11088,7 +11185,7 @@
       </c>
       <c r="E190" s="30" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F190" s="30" t="inlineStr">
@@ -11104,17 +11201,17 @@
       <c r="H190" s="30" t="n"/>
       <c r="I190" s="30" t="inlineStr">
         <is>
-          <t>markets/commoditydetail</t>
+          <t>market/commodity/[key]</t>
         </is>
       </c>
       <c r="J190" s="30" t="inlineStr">
         <is>
-          <t>Live prices only (app/market/commodities.tsx): gold and silver are world prices converted at a live USD/INR, not MCX; unavailable when no live rate.</t>
+          <t>portfolio-analytics.md: gold, silver, crude, natural gas with history; chart is world futures in USD (the rupee card stays labelled as converted, not MCX); futures roll jumps appear. Not verified on a device.</t>
         </is>
       </c>
       <c r="K190" s="30" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -11141,7 +11238,7 @@
       </c>
       <c r="E191" s="30" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F191" s="30" t="inlineStr">
@@ -11157,17 +11254,17 @@
       <c r="H191" s="30" t="n"/>
       <c r="I191" s="30" t="inlineStr">
         <is>
-          <t>markets/forexdetail</t>
+          <t>market/fx/[pair]</t>
         </is>
       </c>
       <c r="J191" s="30" t="inlineStr">
         <is>
-          <t>Live rates only (app/market/fx.tsx): no detail page or history.</t>
+          <t>portfolio-analytics.md: USD/EUR/GBP/JPY/AED to INR with history and a two-way converter at the market rate; JPY chart is stepped (backend rounding). Not verified on a device.</t>
         </is>
       </c>
       <c r="K191" s="30" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -11390,7 +11487,7 @@
       </c>
       <c r="E196" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F196" s="30" t="inlineStr">
@@ -11406,13 +11503,17 @@
       <c r="H196" s="30" t="n"/>
       <c r="I196" s="30" t="inlineStr">
         <is>
-          <t>markets/market-visualizer</t>
-        </is>
-      </c>
-      <c r="J196" s="30" t="n"/>
+          <t>market/map</t>
+        </is>
+      </c>
+      <c r="J196" s="30" t="inlineStr">
+        <is>
+          <t>portfolio-analytics.md: the website deep-dive needs a port-5000 service and scrapes metrics with invented defaults, so it is not ported. Built a different honest visual: Market map (index and sector tiles, 50 large companies by size, coloured by day move). Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K196" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -11492,7 +11593,7 @@
       </c>
       <c r="E198" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F198" s="30" t="inlineStr">
@@ -11508,13 +11609,17 @@
       <c r="H198" s="30" t="n"/>
       <c r="I198" s="30" t="inlineStr">
         <is>
-          <t>markets/options-intelligence</t>
-        </is>
-      </c>
-      <c r="J198" s="30" t="n"/>
+          <t>market/options</t>
+        </is>
+      </c>
+      <c r="J198" s="30" t="inlineStr">
+        <is>
+          <t>portfolio-analytics.md: Black-Scholes price and Greeks (parity-tested against the page's functions), expiry payoff for six strategies from typed strikes and premiums; Nifty spot and India VIX shown for reference. No option chain or IV rank: the page's are random numbers. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K198" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -11541,7 +11646,7 @@
       </c>
       <c r="E199" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F199" s="30" t="inlineStr">
@@ -11560,10 +11665,14 @@
           <t>markets/quantedge</t>
         </is>
       </c>
-      <c r="J199" s="30" t="n"/>
+      <c r="J199" s="30" t="inlineStr">
+        <is>
+          <t>portfolio-analytics.md: the page is hard-coded (72% "edge", fixed radar values) with no model or data behind it. Not built, deliberately. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K199" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -11590,7 +11699,7 @@
       </c>
       <c r="E200" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F200" s="30" t="inlineStr">
@@ -11606,13 +11715,17 @@
       <c r="H200" s="30" t="n"/>
       <c r="I200" s="30" t="inlineStr">
         <is>
-          <t>markets/hedgefund</t>
-        </is>
-      </c>
-      <c r="J200" s="30" t="n"/>
+          <t>portfolio/risk</t>
+        </is>
+      </c>
+      <c r="J200" s="30" t="inlineStr">
+        <is>
+          <t>portfolio-analytics.md: portfolio risk metrics from real history (volatility, worst fall, Calmar, Ulcer, Sharpe, Sortino, beta, tracking error, IR) plus the page's calculators on your own numbers. The page's invented "trading DNA", override cost and BLOCK/TRADE verdicts are not ported. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K200" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -11692,7 +11805,7 @@
       </c>
       <c r="E202" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F202" s="30" t="inlineStr">
@@ -11711,10 +11824,14 @@
           <t>markets/ca-advisor</t>
         </is>
       </c>
-      <c r="J202" s="30" t="n"/>
+      <c r="J202" s="30" t="inlineStr">
+        <is>
+          <t>portfolio-analytics.md: the page is a mock-up (random access codes, a pre-filled fake advisor, buttons that do nothing); real sharing would need a server-side sharing and permissions service that does not exist. The real part (tax dossier) is the phone's Report / ITR tools. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K202" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -11955,7 +12072,7 @@
       </c>
       <c r="E207" s="30" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F207" s="30" t="inlineStr">
@@ -11971,17 +12088,17 @@
       <c r="H207" s="30" t="n"/>
       <c r="I207" s="30" t="inlineStr">
         <is>
-          <t>components/XirrCard.tsx</t>
+          <t>portfolio/sectors</t>
         </is>
       </c>
       <c r="J207" s="30" t="inlineStr">
         <is>
-          <t>XIRR from entered purchase dates done. Sector heatmap / treemap need a sector mapping source and are not built</t>
+          <t>portfolio-analytics.md: XIRR (earlier) plus sector heatmap and treemap from Yahoo's sector names; unmapped stocks are "Unmapped", funds are one bucket, no-price holdings are grey not 0%. HHI and effective N ported. Web preview only. Not verified on a device.</t>
         </is>
       </c>
       <c r="K207" s="30" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12008,7 +12125,7 @@
       </c>
       <c r="E208" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F208" s="30" t="inlineStr">
@@ -12024,13 +12141,17 @@
       <c r="H208" s="30" t="n"/>
       <c r="I208" s="30" t="inlineStr">
         <is>
-          <t>portfolio/quant</t>
-        </is>
-      </c>
-      <c r="J208" s="30" t="n"/>
+          <t>portfolio/simulate, portfolio/risk</t>
+        </is>
+      </c>
+      <c r="J208" s="30" t="inlineStr">
+        <is>
+          <t>portfolio-analytics.md: seeded Monte Carlo cone from assumptions you type (placeholders labelled) and a one-factor (market) regression vs Nifty 50. Multi-factor (Fama-French) not built: no published Indian factor returns; the website's version is estimated from sector composition, not a regression. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K208" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12057,7 +12178,7 @@
       </c>
       <c r="E209" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F209" s="30" t="inlineStr">
@@ -12076,10 +12197,14 @@
           <t>portfolio/research</t>
         </is>
       </c>
-      <c r="J209" s="30" t="n"/>
+      <c r="J209" s="30" t="inlineStr">
+        <is>
+          <t>portfolio-analytics.md: news matched to holdings with the feed's own sentiment labels, valuation table (P/E, P/B, EPS), opt-in peers. Promoter trend NOT built: no shareholding source, and the website table is hard-coded and a quarter old. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K209" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12122,17 +12247,17 @@
       <c r="H210" s="30" t="n"/>
       <c r="I210" s="30" t="inlineStr">
         <is>
-          <t>app/tracker/watchlist.tsx</t>
+          <t>market/screener</t>
         </is>
       </c>
       <c r="J210" s="30" t="inlineStr">
         <is>
-          <t>Watchlist done (price at add, honest offline). Screener needs a backend and is not built</t>
+          <t>portfolio-analytics.md: watchlist (earlier) plus screener filters on backend fundamentals (sector, P/E, P/B, the Deep Value rule, parity-tested; a missing figure never passes). Presets needing ROE, debt/equity, dividend yield, revenue growth are not built (no data). Not verified on a device.</t>
         </is>
       </c>
       <c r="K210" s="30" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12208,7 +12333,7 @@
       </c>
       <c r="E212" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F212" s="30" t="inlineStr">
@@ -12229,12 +12354,12 @@
       </c>
       <c r="J212" s="30" t="inlineStr">
         <is>
-          <t>Standalone app; own sync via a vault id</t>
+          <t>trade-journal.md: log, edit, analytics, psychology as counts only, CSV / broker trade book / website-backup import with preview, dedupe and undo, CSV export. Device-only from cloud sync (finos_sync_never_ prefix). OCR scan of broker screenshots NOT built (needs an OCR dependency or backend and a privacy decision). Broker file formats untested on real files. Many website analytics (Sharpe, Kelly, VaR, scores, XP) deliberately not ported. Not verified on a device.</t>
         </is>
       </c>
       <c r="K212" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12261,7 +12386,7 @@
       </c>
       <c r="E213" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F213" s="30" t="inlineStr">
@@ -12282,12 +12407,12 @@
       </c>
       <c r="J213" s="30" t="inlineStr">
         <is>
-          <t>Separate Vite+Express service; npm advisories open</t>
+          <t>The headlines part is on the phone: app/market/news.tsx (see M-19) via the arya-ai backend's news route, with an honest offline state. The separate News1 app (Vite + Express service, its own sources and npm advisories) is not ported.</t>
         </is>
       </c>
       <c r="K213" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12367,7 +12492,7 @@
       </c>
       <c r="E215" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F215" s="30" t="inlineStr">
@@ -12388,12 +12513,12 @@
       </c>
       <c r="J215" s="30" t="inlineStr">
         <is>
-          <t>Ranking: js/arya-pulse-rank.js</t>
+          <t>arya-tabs.md: the website has 27 ranked widgets (not 24); 17 are on the phone (added net worth timeline, wealth velocity from an on-device history, Monte Carlo "will my money last"); 10 are left out with a reason each (assumption-driven or no source), listed in lib/pulseCards.ts. Not verified on a device.</t>
         </is>
       </c>
       <c r="K215" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12420,7 +12545,7 @@
       </c>
       <c r="E216" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F216" s="30" t="inlineStr">
@@ -12436,13 +12561,17 @@
       <c r="H216" s="30" t="n"/>
       <c r="I216" s="30" t="inlineStr">
         <is>
-          <t>arya/plan</t>
-        </is>
-      </c>
-      <c r="J216" s="30" t="n"/>
+          <t>arya/plan, arya/map, arya/life</t>
+        </is>
+      </c>
+      <c r="J216" s="30" t="inlineStr">
+        <is>
+          <t>arya-tabs.md: Plan (8 steps, "needs a figure" when unrecorded), Map (allocation from recorded assets), Life (timeline of declared events and goal dates). No assumed income, age or return. Website age-benchmark targets not built. Web preview only. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K216" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12469,7 +12598,7 @@
       </c>
       <c r="E217" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F217" s="30" t="inlineStr">
@@ -12485,13 +12614,17 @@
       <c r="H217" s="30" t="n"/>
       <c r="I217" s="30" t="inlineStr">
         <is>
-          <t>arya/agent</t>
-        </is>
-      </c>
-      <c r="J217" s="30" t="n"/>
+          <t>arya/cal, arya/india, arya/agent</t>
+        </is>
+      </c>
+      <c r="J217" s="30" t="inlineStr">
+        <is>
+          <t>arya-tabs.md: Cal (upcoming dates, 26-week spending heatmap), India (income-tax rules with source and year; the website's unsourced state cost-of-life map is NOT ported), Agent (tool loop screen). Rules are FY 2025-26 as coded; the screen warns when today's FY is later. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K217" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12518,7 +12651,7 @@
       </c>
       <c r="E218" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F218" s="30" t="inlineStr">
@@ -12539,12 +12672,12 @@
       </c>
       <c r="J218" s="30" t="inlineStr">
         <is>
-          <t>Backend tools exist; phone has no tool loop</t>
+          <t>arya-tabs.md: a visible phone tool loop with 44 tools (recorded figures, calculator hub, public lookups); every call is listed, results carry source and time, off switch. A model-chosen tool loop is NOT built (needs native tool calling on /api/chat) and personas and run history are not built. Not verified on a device.</t>
         </is>
       </c>
       <c r="K218" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12571,7 +12704,7 @@
       </c>
       <c r="E219" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F219" s="30" t="inlineStr">
@@ -12590,10 +12723,14 @@
           <t>arya/memory</t>
         </is>
       </c>
-      <c r="J219" s="30" t="n"/>
+      <c r="J219" s="30" t="inlineStr">
+        <is>
+          <t>Verified; chat can now write a note through the memory store's refusal rules, the Life tab shows life events with what each changes. Switches default off. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K219" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12696,12 +12833,12 @@
       </c>
       <c r="J221" s="30" t="inlineStr">
         <is>
-          <t>Mic permission is declared in app.json; no feature built</t>
+          <t>Not built. The microphone permission is not declared: RECORD_AUDIO is blocked in app.json and a test fails if a microphone, speech or camera permission returns (R-17).</t>
         </is>
       </c>
       <c r="K221" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -12728,7 +12865,7 @@
       </c>
       <c r="E222" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Not planned</t>
         </is>
       </c>
       <c r="F222" s="30" t="inlineStr">
@@ -12747,10 +12884,14 @@
           <t>arya/</t>
         </is>
       </c>
-      <c r="J222" s="30" t="n"/>
+      <c r="J222" s="30" t="inlineStr">
+        <is>
+          <t>arya-tabs.md: Money AI page = the Arya tab (A-01); the chatbot brain is a server-side proxy the phone already reaches through /api/chat; RAG filings cannot be honest because no NSE/BSE filings are indexed (only regulation and FIN-OS page documents). Backend request in docs/PENDING.md U14. Not verified on a device.</t>
+        </is>
+      </c>
       <c r="K222" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -13063,12 +13204,12 @@
       </c>
       <c r="J228" s="30" t="inlineStr">
         <is>
-          <t>Planner unit-tested (11 cases); permission flow + OS scheduling built but NOT verified on a device (needs R-08/R-09). Local only, no push token.</t>
+          <t>Planner unit-tested (11 cases); the explain-first permission flow (lib/permissions.ts, permissionPrompt) and OS scheduling are built but NOT verified on a device (needs R-08/R-09; checklist rows D-20..D-26). Local only, no push token; scheduled and delivered notices are cleared by Erase.</t>
         </is>
       </c>
       <c r="K228" s="30" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -13095,7 +13236,7 @@
       </c>
       <c r="E229" s="30" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F229" s="30" t="inlineStr">
@@ -13116,12 +13257,12 @@
       </c>
       <c r="J229" s="30" t="inlineStr">
         <is>
-          <t>Nudges done (only from recorded facts, dismissible). Persona greetings and the status strip not built</t>
+          <t>Home (app/(tabs)/dashboard.tsx, lib/persona.ts, components/PersonaStrip.tsx): time-of-day greeting with the first name only when one is recorded (no stand-in name), 'N-day streak' from day two, and a strip of savings rate, net worth and Money Score, each only when recorded; the cross hides it and Settings brings it back (finos_persona_mobile, device-only). Nudges as before. An honest subset of FinosPersona: left out on purpose are the Financial DNA archetype and life-stage labels, the Health score chip (it rests on a neutral DNA baseline and a 60,000 income fallback), FIRE % and the trade-journal win rate. Web preview only, not a device.</t>
         </is>
       </c>
       <c r="K229" s="30" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -13871,12 +14012,12 @@
       <c r="I244" s="30" t="n"/>
       <c r="J244" s="30" t="inlineStr">
         <is>
-          <t>App side built and tested (erase phone, delete cloud copy, delete account via RPC). Needs supabase/delete_account.sql run on the live project before 'Delete my account' works.</t>
+          <t>App side built and tested: one erase flow (signs out first, clears memory, notifications, cache files, secure storage, then checks for leftovers), delete the cloud copy, delete account via RPC. supabase/delete_account.sql now also deletes the rows of tables with no cascade (alerts, push_subscriptions, alert_preferences, health_score_history, memory_embeddings, user_behavior, document_ai_log, couple links), guarded by a test and proved in a throwaway PostgreSQL (scripts/release-sql-check.py), but NOT run on the live project. Owner decision open: deleting a couple link also removes the partner's shared goals.</t>
         </is>
       </c>
       <c r="K244" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -14020,12 +14161,12 @@
       <c r="I247" s="30" t="n"/>
       <c r="J247" s="30" t="inlineStr">
         <is>
-          <t>Everything so far ran in the web preview</t>
+          <t>Everything so far ran in the web preview. docs/DEVICE_TEST_CHECKLIST.md lists what needs a phone (sections A-I); no row has been run.</t>
         </is>
       </c>
       <c r="K247" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -14073,12 +14214,12 @@
       </c>
       <c r="J248" s="30" t="inlineStr">
         <is>
-          <t>Planner unit-tested (11 cases); permission flow + OS scheduling built but NOT verified on a device (needs R-08/R-09). Local only, no push token.</t>
+          <t>Explain-first flow built for reminders and the biometric switch (the OS prompt appears only after the person agrees on our screen); planner unit-tested; denial path shows a plain message and the switch does not claim 'on'. NOT verified on a device (needs R-08/R-09; checklist rows D-20..D-24).</t>
         </is>
       </c>
       <c r="K248" s="30" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -14105,7 +14246,7 @@
       </c>
       <c r="E249" s="30" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F249" s="30" t="inlineStr">
@@ -14122,12 +14263,12 @@
       <c r="I249" s="30" t="n"/>
       <c r="J249" s="30" t="inlineStr">
         <is>
-          <t>Placeholders only</t>
+          <t>Built: icon, adaptive icon (with monochrome layer), splash, notification icon, Play 512 icon and feature graphic (mobile/scripts/release-assets.py, reproducible, tested for size, alpha and safe zones), 28 store screenshots from the web preview with a synthetic profile (not device captures, taken before the Oct 17 Budget / Goals clipping fix), and listing text in docs/STORE_LISTING.md. Not done: legal operator and URLs, store accounts and forms, screenshots from a device (all need the owner; PENDING U6/U7).</t>
         </is>
       </c>
       <c r="K249" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -14224,12 +14365,12 @@
       <c r="I251" s="30" t="n"/>
       <c r="J251" s="30" t="inlineStr">
         <is>
-          <t>On-device redacted crash notes, error boundary, Diagnostics screen and opt-in screen counts (default off); nothing is sent automatically and there is no crash service. Fatal native crashes may kill the process before a note is written.</t>
+          <t>On-device redacted crash notes, error boundary, Diagnostics screen and opt-in screen counts (default off); nothing is sent automatically and there is no crash service. Fatal native crashes may kill the process before a note is written. Play Android vitals and App Store Connect remain the only automatic crash signals. Not run on a device.</t>
         </is>
       </c>
       <c r="K251" s="30" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -14381,12 +14522,12 @@
       <c r="I254" s="30" t="n"/>
       <c r="J254" s="30" t="inlineStr">
         <is>
-          <t>Needs the user's Supabase dashboard login</t>
+          <t>Needs the user's Supabase dashboard login. The file has been rewritten (see R-06) and passes its guard test; it has not been run on any project.</t>
         </is>
       </c>
       <c r="K254" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -14435,7 +14576,7 @@
       </c>
       <c r="K255" s="30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-17</t>
         </is>
       </c>
     </row>
@@ -15204,7 +15345,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="12" customWidth="1" style="16" min="1" max="1"/>
@@ -16078,6 +16219,342 @@
       </c>
       <c r="E33" s="16" t="n">
         <v>359</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>L-01..L-26, T-36</t>
+        </is>
+      </c>
+      <c r="C34" s="16" t="inlineStr">
+        <is>
+          <t>Learn: 25 lessons bundled in the app with on-device progress, search entries, Knowledge pillar follows the website</t>
+        </is>
+      </c>
+      <c r="D34" s="16" t="inlineStr">
+        <is>
+          <t>Per docs/agent-notes/learn.md: learn.test.mts (14) incl. a golden test against js/finos-health-score.js; preview run. Logged here on 2026-10-17 from the agent note; not re-run line by line</t>
+        </is>
+      </c>
+      <c r="E34" s="16" t="n">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>T-19, M-21</t>
+        </is>
+      </c>
+      <c r="C35" s="16" t="inlineStr">
+        <is>
+          <t>Insurance hub (cover types, questions, your policies beside them) and mutual-fund search, detail and compare</t>
+        </is>
+      </c>
+      <c r="D35" s="16" t="inlineStr">
+        <is>
+          <t>Per docs/agent-notes/insurance-mf.md: parity with js/mf-intelligence.js, extraction script check; preview run. Logged from the note</t>
+        </is>
+      </c>
+      <c r="E35" s="16" t="n">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>A-02, A-05, A-06</t>
+        </is>
+      </c>
+      <c r="C36" s="16" t="inlineStr">
+        <is>
+          <t>PULSE feed (14 of 27 widgets), Arya memory and life events, local Arya tools</t>
+        </is>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>Per docs/agent-notes/arya-pulse.md: ranking vs js/arya-pulse-rank.js on 600 contexts, 33 positive + 15 negative intent phrases; preview run. Logged from the note</t>
+        </is>
+      </c>
+      <c r="E36" s="16" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>M-04, M-05, M-06, M-15, M-19</t>
+        </is>
+      </c>
+      <c r="C37" s="16" t="inlineStr">
+        <is>
+          <t>Market research: stock and fund detail, screener, news with stated sentiment, commodities, FX, crypto lists; offline cache with time</t>
+        </is>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>Per docs/agent-notes/market-data.md: marketData tests (33) + backend pytest (30, stubs only); preview run. Logged from the note</t>
+        </is>
+      </c>
+      <c r="E37" s="16" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>T-01, T-02, T-10, T-18, T-38, T-39</t>
+        </is>
+      </c>
+      <c r="C38" s="16" t="inlineStr">
+        <is>
+          <t>Growth projection, spending forecast, life goals planner, couple finance, benchmarks, your own calendar dates</t>
+        </is>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>Per docs/agent-notes/planners.md: parity vs the website cores, mutation checks, smoke 6 screens x 4 runs = 0; theme audit 0 low-contrast. Logged from the note</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>P-08, P-11, R-06, R-10, R-13, P-10</t>
+        </is>
+      </c>
+      <c r="C39" s="16" t="inlineStr">
+        <is>
+          <t>Trust platform: onboarding, feedback, crash notes, erase flow, explain-first permissions, lock hardening, Google sign-in code path (hidden)</t>
+        </is>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>Per docs/agent-notes/trust-platform.md: redaction and feedback parity, erase and lock tests, mutation checks. Google sign-in unit-tested with fakes only. Logged from the note</t>
+        </is>
+      </c>
+      <c r="E39" s="16" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>R-11, R-17</t>
+        </is>
+      </c>
+      <c r="C40" s="16" t="inlineStr">
+        <is>
+          <t>Release pack: brand assets, store screenshots, release config guards, store copy, runbook, SQL harness</t>
+        </is>
+      </c>
+      <c r="D40" s="16" t="inlineStr">
+        <is>
+          <t>Per docs/agent-notes/release-pack.md: releaseAssets (7) + releaseConfig (11) tests; SQL run in a throwaway PostgreSQL 16. Logged from the note</t>
+        </is>
+      </c>
+      <c r="E40" s="16" t="n">
+        <v>676</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B41" s="16" t="inlineStr">
+        <is>
+          <t>(robustness, no row)</t>
+        </is>
+      </c>
+      <c r="C41" s="16" t="inlineStr">
+        <is>
+          <t>Stored and received data of the wrong shape never crashes a screen or becomes NaN; a failed read is never saved over data; backup restore all-or-nothing</t>
+        </is>
+      </c>
+      <c r="D41" s="16" t="inlineStr">
+        <is>
+          <t>Per docs/agent-notes/mobile-robustness.md: corruptData.test.mts (170) with four mutation checks; corrupt-data web smoke over every route x 5 variants = 0</t>
+        </is>
+      </c>
+      <c r="E41" s="16" t="n">
+        <v>846</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>P-07, R-11, R-06, A-02, A-05, A-06</t>
+        </is>
+      </c>
+      <c r="C42" s="16" t="inlineStr">
+        <is>
+          <t>Cross-links (Budget to Forecast, Goals to Life goals, Portfolio to Growth, Insurance to hub, Watchlist rows to research, feedback on the Money Score); Home facts strip and honest greeting; assumed ages removed; Budget / Goals input clipping and Portfolio title wrap fixed; privacy line for kept-aside values; Hindi first pass; tracker rows audited against the code</t>
+        </is>
+      </c>
+      <c r="D42" s="16" t="inlineStr">
+        <is>
+          <t>persona.test.mts (new), privacy and logic tests extended with mutation checks; tsc clean; Playwright run of each new link at 430 px; smoke-routes and theme-audit on the changed screens (see docs/agent-notes/mobile-polish.md). Web preview only, nothing on a device</t>
+        </is>
+      </c>
+      <c r="E42" s="16" t="inlineStr">
+        <is>
+          <t>952</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>L-22, L-24..L-51</t>
+        </is>
+      </c>
+      <c r="C43" s="16" t="inlineStr">
+        <is>
+          <t>Learn wave 2: 5 new lessons (mindset-sim case studies, impact stories, decision, clarity, life-wealth), line provenance on every quoted passage, honest stub pages for the 22 interactive website pages (hub / redirect / not on the phone, each with its reason). Merged from docs/agent-notes/learn2.md.</t>
+        </is>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>learn2.test.mts (9), learn.test.mts; extract-learn.py --check; smoke on the new routes (per the note, not re-run for each)</t>
+        </is>
+      </c>
+      <c r="E43" s="16" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B44" s="16" t="inlineStr">
+        <is>
+          <t>A-02..A-06, A-09</t>
+        </is>
+      </c>
+      <c r="C44" s="16" t="inlineStr">
+        <is>
+          <t>Arya Plan / Map / Life / Cal / India / Agent tabs, 44-tool visible tool loop, PULSE 17 of 27, net-worth history. A-09 not built (reasons). Merged from docs/agent-notes/arya-tabs.md.</t>
+        </is>
+      </c>
+      <c r="D44" s="16" t="inlineStr">
+        <is>
+          <t>aryaIntent, aryaToolbox, aryaServerTools, aryaAgent, aryaTabs tests; smoke 8 screens x 4 runs 0 problems (per the note)</t>
+        </is>
+      </c>
+      <c r="E44" s="16" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>M-07, M-08, M-09, M-14, M-16, M-17, M-18, M-20, S-04..S-07</t>
+        </is>
+      </c>
+      <c r="C45" s="16" t="inlineStr">
+        <is>
+          <t>Crypto / commodity / forex detail with history, Market map, Options calculator, Portfolio analytics (sectors and treemap, risk, simulation, research), screener filters. M-17 and M-20 not built (static placeholders / mock-up). Merged from docs/agent-notes/portfolio-analytics.md.</t>
+        </is>
+      </c>
+      <c r="D45" s="16" t="inlineStr">
+        <is>
+          <t>Parity tests against the website's own functions in a vm (per the note); smoke per the note</t>
+        </is>
+      </c>
+      <c r="E45" s="16" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>S-09</t>
+        </is>
+      </c>
+      <c r="C46" s="16" t="inlineStr">
+        <is>
+          <t>Trade journal: log, analytics, psychology counts, CSV / broker / backup import with undo, export; device-only from sync. OCR not built. Merged from docs/agent-notes/trade-journal.md.</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>tradeJournal (39), tradeJournalImport (12), tradeJournal.parity (20: 12 pass, 8 todo = website defects); mutation checks</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="16" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>(final integration, no row)</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="inlineStr">
+        <is>
+          <t>Shared files: search entries + index guard, privacy notice and data inventory, Hindi first pass, route samples, Home / Portfolio links. Health score no longer computed from no data (Not enough data; only recorded areas scored, missing named). Safe-area insets, screen-title headings, dark purple text, 200% layout fixes. See docs/agent-notes/final-integration.md.</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>npm test + tsc + smoke-routes + theme-audit on a fresh Metro (see the note); nothing on a device</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="n">
+        <v>1057</v>
       </c>
     </row>
   </sheetData>

</xml_diff>